<commit_message>
Fix formula-text conflict in 05_Asset_Depreciation.xlsx: prefix display strings starting with = to prevent openpyxl from treating them as Excel formulas
</commit_message>
<xml_diff>
--- a/rFLA300/chapter-11/05_Asset_Depreciation.xlsx
+++ b/rFLA300/chapter-11/05_Asset_Depreciation.xlsx
@@ -812,9 +812,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="11">
-        <f>SLN(cost, salvage, life)  →  Same amount every year</f>
-        <v/>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =SLN(cost, salvage, life)  →  Same amount every year</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -858,9 +859,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="11">
-        <f>DB(cost, salvage, life, period, [month])  →  Higher depreciation in early years</f>
-        <v/>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =DB(cost, salvage, life, period, [month])  →  Higher depreciation in early years</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -915,9 +917,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="11">
-        <f>DDB(cost, salvage, life, period, [factor])  →  Fastest depreciation; factor=2 by default</f>
-        <v/>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  =DDB(cost, salvage, life, period, [factor])  →  Fastest depreciation; factor=2 by default</t>
+        </is>
       </c>
     </row>
     <row r="25">

</xml_diff>